<commit_message>
Add PET cups tab with Redds quote
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K8tdfK9jnadBsXYfH8huwz
</commit_message>
<xml_diff>
--- a/out/cup_supplier_comparison.xlsx
+++ b/out/cup_supplier_comparison.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PET Cups" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -96,6 +97,7 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1038,4 +1040,213 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PET (clear plastic) cups – separate from the paper cup comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GST rate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Credit card surcharge</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Unit price ex GST</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Shipping ex GST</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Subtotal ex GST</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Total inc GST</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Cost / piece ex GST</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Cost / piece inc GST</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="62" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Redds Custom Printing</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>16oz Clear PET, 1 colour logo, 1 side (direct deposit price)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7">
+        <f>C5*D5+E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="7">
+        <f>F5*$B$2</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>F5+G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
+        <f>F5/C5</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>H5/C5</f>
+        <v/>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Shipping included. Quote total $1,800 ex GST. No lids quoted. PDF is dated January 2025 - confirm the price is still current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Redds Custom Printing</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Same, paying by credit card</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="6">
+        <f>D5*(1+$F$2)</f>
+        <v/>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7">
+        <f>C6*D6+E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="7">
+        <f>F6*$B$2</f>
+        <v/>
+      </c>
+      <c r="H6" s="7">
+        <f>F6+G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="6">
+        <f>F6/C6</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>H6/C6</f>
+        <v/>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Quote says credit card pays the original (higher) price plus a 2% surcharge. The original price isn't shown, so only the 2% is applied here - ask Redds for the card price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Add more PET quotes in the rows below (same columns). Blue = typed inputs, black = formulas.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add lead time column to comparison sheets and CSV
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K8tdfK9jnadBsXYfH8huwz
</commit_message>
<xml_diff>
--- a/out/cup_supplier_comparison.xlsx
+++ b/out/cup_supplier_comparison.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +98,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -478,7 +481,8 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,6 +510,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -569,11 +574,16 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
+          <t>Lead time</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="95" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>Vista Corporate</t>
@@ -623,11 +633,16 @@
       </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
+          <t>Not stated on quote ('production time after payment and artwork/proof approval'). Ask Vista for days</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
           <t>Full colour print, white sip-thru lid. Quote total $10,614.00 inc GST; lid + standard delivery included. Quote dated 27/10/2026, valid 30 days.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="95" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
           <t>bioSupply</t>
@@ -677,13 +692,18 @@
         <f>J6/C6</f>
         <v/>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>Not stated - 'Standard dispatch', clock starts at final artwork approval; account manager confirms date. bioSupply site: ~10 business days standard (ad-hoc orders), express 7-day +25%, 5-day +50%. Confirm for pallet-size runs</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>CMYK front only, 80mm. Lid = stock 90mm lid at $494/10,000 (not priced per size on quote). Freight = TNT email figure, applied only if switch above = 1. Quote BQ-1181 valid to 25 Nov.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="95" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>Vista Corporate</t>
@@ -733,11 +753,16 @@
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
+          <t>Not stated on quote ('production time after payment and artwork/proof approval'). Ask Vista for days</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
           <t>Quote total $18,490.00 inc GST; lid + standard delivery included.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="95" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>bioSupply</t>
@@ -787,13 +812,18 @@
         <f>J8/C8</f>
         <v/>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>Not stated - 'Standard dispatch', clock starts at final artwork approval; account manager confirms date. bioSupply site: ~10 business days standard (ad-hoc orders), express 7-day +25%, 5-day +50%. Confirm for pallet-size runs</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>CMYK front only, 80mm. Lid and freight as above.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="95" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>Vista Corporate</t>
@@ -843,11 +873,16 @@
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
+          <t>Not stated on quote ('production time after payment and artwork/proof approval'). Ask Vista for days</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
           <t>Quote total $7,876.00 inc GST; lid + standard delivery included.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="95" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
           <t>bioSupply</t>
@@ -896,12 +931,18 @@
         <f>J10/C10</f>
         <v/>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>Not stated - 'Standard dispatch', clock starts at final artwork approval; account manager confirms date. bioSupply site: ~10 business days standard (ad-hoc orders), express 7-day +25%, 5-day +50%. Confirm for pallet-size runs</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>Only 10,000 quoted (Vista is 20,000). Delivery included on quote; no TNT freight given for 16oz.</t>
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
@@ -988,6 +1029,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
@@ -1048,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1061,7 +1103,8 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1089,6 +1132,7 @@
         <v>0.02</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1142,6 +1186,11 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
+          <t>Lead time</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -1188,6 +1237,11 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
+          <t>Not stated on the Redds quote. Ask print@reddcups.com.au for production days after artwork approval</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
           <t>Shipping included. Quote total $1,800 ex GST. No lids quoted. PDF is dated January 2025 - confirm the price is still current.</t>
         </is>
       </c>
@@ -1235,10 +1289,16 @@
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
+          <t>Not stated on the Redds quote. Ask print@reddcups.com.au for production days after artwork approval</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
           <t>Quote says credit card pays the original (higher) price plus a 2% surcharge. The original price isn't shown, so only the 2% is applied here - ask Redds for the card price.</t>
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>

</xml_diff>